<commit_message>
Fixed basic solver issues not accounting for fatiuge Fixed placement of entrance and pivot accomidation for excel
</commit_message>
<xml_diff>
--- a/tests/Full Shift Test/test file 1.xlsx
+++ b/tests/Full Shift Test/test file 1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Weekly_Grid" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="75">
   <si>
     <t xml:space="preserve">job name</t>
   </si>
@@ -209,12 +209,6 @@
   </si>
   <si>
     <t xml:space="preserve">Officer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sol1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sol2</t>
   </si>
   <si>
     <t xml:space="preserve">required talents</t>
@@ -1426,27 +1420,9 @@
         <v>61</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>43</v>
-      </c>
+      <c r="A28" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1475,24 +1451,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>67</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>69</v>
       </c>
       <c r="E2" s="3"/>
     </row>
@@ -1504,30 +1480,30 @@
         <v>43</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>43</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1538,7 +1514,7 @@
         <v>43</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E6" s="3"/>
     </row>
@@ -1547,10 +1523,10 @@
         <v>25</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1558,10 +1534,10 @@
         <v>26</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E8" s="3"/>
     </row>
@@ -1661,10 +1637,10 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>